<commit_message>
Updated using government land-use data
</commit_message>
<xml_diff>
--- a/InputData/land/BLAPE/BAU LULUCF Anthro Pollutant Emis.xlsx
+++ b/InputData/land/BLAPE/BAU LULUCF Anthro Pollutant Emis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Postdoc Projects/eps-indonesia-cpl/InputData/land/BLAPE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA7D5D32-E1E0-D84B-BD61-DE1144AF335A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1CF161F-5235-DC43-9FE3-FDC7489E1C16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21380" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21360" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -1394,7 +1394,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="51"/>
                 <c:pt idx="0">
-                  <c:v>376</c:v>
+                  <c:v>336</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>326</c:v>
@@ -7623,7 +7623,7 @@
         <v>818.65</v>
       </c>
       <c r="V12">
-        <v>376</v>
+        <v>336</v>
       </c>
       <c r="W12">
         <v>326</v>
@@ -8690,7 +8690,7 @@
       </c>
       <c r="B21">
         <f>V12</f>
-        <v>376</v>
+        <v>336</v>
       </c>
       <c r="C21">
         <f t="shared" ref="C21:D21" si="43">W12</f>
@@ -10998,7 +10998,7 @@
       </c>
       <c r="B81">
         <f>B21</f>
-        <v>376</v>
+        <v>336</v>
       </c>
       <c r="C81">
         <f t="shared" ref="C81:AZ81" si="46">C21</f>
@@ -11415,7 +11415,7 @@
       </c>
       <c r="B2" s="37">
         <f>'GWF-Smoothing '!B81</f>
-        <v>376</v>
+        <v>336</v>
       </c>
       <c r="C2" s="37">
         <f>'GWF-Smoothing '!C81</f>
@@ -11720,10 +11720,10 @@
       </c>
       <c r="B4" s="37">
         <f>B2*$B$3</f>
-        <v>376000000</v>
+        <v>336000000</v>
       </c>
       <c r="C4" s="37">
-        <f t="shared" ref="C4:BN4" si="0">C2*$B$3</f>
+        <f t="shared" ref="C4:AZ4" si="0">C2*$B$3</f>
         <v>326000000</v>
       </c>
       <c r="D4" s="37">
@@ -11948,7 +11948,7 @@
       </c>
       <c r="B5" s="29">
         <f>B4*'Share of Pollutants'!$B$19</f>
-        <v>220447809.08522567</v>
+        <v>196995914.50169101</v>
       </c>
       <c r="C5" s="29">
         <f>C4*'Share of Pollutants'!$B$19</f>
@@ -12176,7 +12176,7 @@
       </c>
       <c r="B6" s="29">
         <f>B4*'Share of Pollutants'!$B$20</f>
-        <v>95548758.043509468</v>
+        <v>85383996.549519092</v>
       </c>
       <c r="C6" s="29">
         <f>C4*'Share of Pollutants'!$B$20</f>
@@ -12404,7 +12404,7 @@
       </c>
       <c r="B7" s="29">
         <f>B4*'Share of Pollutants'!$B$21</f>
-        <v>60003432.871264853</v>
+        <v>53620088.948789872</v>
       </c>
       <c r="C7" s="29">
         <f>C4*'Share of Pollutants'!$B$21</f>
@@ -12855,10 +12855,10 @@
       </c>
       <c r="B11" s="29">
         <f>B5*$B$8</f>
-        <v>220447809085225.66</v>
+        <v>196995914501691</v>
       </c>
       <c r="C11" s="29">
-        <f t="shared" ref="C11:BN12" si="1">C5*$B$8</f>
+        <f t="shared" ref="C11:AZ12" si="1">C5*$B$8</f>
         <v>191132940855807.38</v>
       </c>
       <c r="D11" s="29">
@@ -13083,7 +13083,7 @@
       </c>
       <c r="B12" s="29">
         <f t="shared" ref="B12:Q13" si="2">B6*$B$8</f>
-        <v>95548758043509.469</v>
+        <v>85383996549519.094</v>
       </c>
       <c r="C12" s="29">
         <f t="shared" si="2"/>
@@ -13311,10 +13311,10 @@
       </c>
       <c r="B13" s="29">
         <f t="shared" si="2"/>
-        <v>60003432871264.852</v>
+        <v>53620088948789.875</v>
       </c>
       <c r="C13" s="29">
-        <f t="shared" ref="C13:BN13" si="3">C7*$B$8</f>
+        <f t="shared" ref="C13:AZ13" si="3">C7*$B$8</f>
         <v>52024252968171.117</v>
       </c>
       <c r="D13" s="29">
@@ -13612,10 +13612,10 @@
       </c>
       <c r="B15" s="29">
         <f>B11/$B$22</f>
-        <v>220447809085225.66</v>
+        <v>196995914501691</v>
       </c>
       <c r="C15" s="29">
-        <f t="shared" ref="C15:BN15" si="4">C11/$B$22</f>
+        <f t="shared" ref="C15:AZ15" si="4">C11/$B$22</f>
         <v>191132940855807.38</v>
       </c>
       <c r="D15" s="29">
@@ -13840,10 +13840,10 @@
       </c>
       <c r="B16" s="29">
         <f>B12/$B$23</f>
-        <v>3412455644411.0522</v>
+        <v>3049428448197.1104</v>
       </c>
       <c r="C16" s="29">
-        <f t="shared" ref="C16:BN16" si="5">C12/$B$23</f>
+        <f t="shared" ref="C16:AZ16" si="5">C12/$B$23</f>
         <v>2958671649143.625</v>
       </c>
       <c r="D16" s="29">
@@ -14068,10 +14068,10 @@
       </c>
       <c r="B17" s="29">
         <f>B13/$B$24</f>
-        <v>226428048570.81076</v>
+        <v>202339958297.32028</v>
       </c>
       <c r="C17" s="29">
-        <f t="shared" ref="C17:BN17" si="6">C13/$B$24</f>
+        <f t="shared" ref="C17:AZ17" si="6">C13/$B$24</f>
         <v>196317935728.9476</v>
       </c>
       <c r="D17" s="29">
@@ -15355,7 +15355,7 @@
       </c>
       <c r="B2" s="24">
         <f>'Global Watch Data'!B15</f>
-        <v>220447809085225.66</v>
+        <v>196995914501691</v>
       </c>
       <c r="C2" s="24">
         <f>'Global Watch Data'!C15</f>
@@ -16828,7 +16828,7 @@
       </c>
       <c r="B11" s="27">
         <f>'Global Watch Data'!B16</f>
-        <v>3412455644411.0522</v>
+        <v>3049428448197.1104</v>
       </c>
       <c r="C11" s="27">
         <f>'Global Watch Data'!C16</f>
@@ -17037,7 +17037,7 @@
       </c>
       <c r="B12" s="27">
         <f>'Global Watch Data'!B17</f>
-        <v>226428048570.81076</v>
+        <v>202339958297.32028</v>
       </c>
       <c r="C12" s="27">
         <f>'Global Watch Data'!C17</f>

</xml_diff>

<commit_message>
Updated PEREC and Average distance travelled
</commit_message>
<xml_diff>
--- a/InputData/land/BLAPE/BAU LULUCF Anthro Pollutant Emis.xlsx
+++ b/InputData/land/BLAPE/BAU LULUCF Anthro Pollutant Emis.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Postdoc Projects/eps-indonesia-cpl/InputData/land/BLAPE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1CF161F-5235-DC43-9FE3-FDC7489E1C16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C54440B6-3C19-984A-89B4-6C13699EAB59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21360" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>